<commit_message>
docs(eval): refresh AI platform radar
</commit_message>
<xml_diff>
--- a/outputs/01a05ade-6b8d-7f02-bfaa-2d4e3f2df08c/novelAssist-dsh-项目评估图谱-2026-09-01.xlsx
+++ b/outputs/01a05ade-6b8d-7f02-bfaa-2d4e3f2df08c/novelAssist-dsh-项目评估图谱-2026-09-01.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_总览" sheetId="1" r:id="R1e14a6ab03714f93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_模块成熟度" sheetId="2" r:id="Rf21aa3c13744459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_能力闭环" sheetId="3" r:id="Rbfe5d150e1ee464f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_上下文与复用" sheetId="4" r:id="Rb476685302344dae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_LLM调用点" sheetId="5" r:id="R98dabe6c0c864b95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_AI平台" sheetId="6" r:id="R3f201417909540d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_模型适配" sheetId="7" r:id="Rf32435e74dbc42e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_评测计划" sheetId="8" r:id="R47418c1564df41b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_路线图" sheetId="9" r:id="R1bd50dfa551d405f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_证据索引" sheetId="10" r:id="Rc9646ad37e4f4455"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_评分规则" sheetId="11" r:id="R76677866addd4cf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_总览" sheetId="1" r:id="R4621ce1a03504f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_模块成熟度" sheetId="2" r:id="Rc75ed8582edc4fda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_能力闭环" sheetId="3" r:id="R777797a505fd4428"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_上下文与复用" sheetId="4" r:id="Raaa761b396724d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_LLM调用点" sheetId="5" r:id="R75b7b1c94e494b4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_AI平台" sheetId="6" r:id="R73cc4d63fff94eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_模型适配" sheetId="7" r:id="R78e5fc8985b14b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_评测计划" sheetId="8" r:id="Rcd2fdf097dc24825"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_路线图" sheetId="9" r:id="Rd288e1e01518464d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_证据索引" sheetId="10" r:id="Rb35942b44fd542d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_评分规则" sheetId="11" r:id="Ree6eb8c56e754fda"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -85,7 +85,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -145,6 +145,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFB91C1C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9F0F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -274,7 +284,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="194">
+  <x:cellXfs count="198">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -749,6 +759,18 @@
     <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="13" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="14" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -760,7 +782,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -771,7 +793,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -782,7 +804,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECFDF3"/>
         </x:patternFill>
       </x:fill>
@@ -793,7 +815,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -804,7 +826,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -815,7 +837,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -826,7 +848,7 @@
         <x:color rgb="FF2563EB"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF2FF"/>
         </x:patternFill>
       </x:fill>
@@ -981,7 +1003,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45eff83e570a4482"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0ef5feea110f40da"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2385,7 +2407,7 @@
     <x:mergeCell ref="A29:H32"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b26640d27d247fc"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R959c6558c14e422f"/>
 </x:worksheet>
 </file>
 
@@ -3153,7 +3175,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red13a4410f424b24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ea0735b21cd4f71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4761,7 +4783,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54a00741c08145ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12a11d8fe0a7422e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5981,7 +6003,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1f882a6bd214c69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R432376c739154f6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6596,8 +6618,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd219f4fa0e694ec6"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c7eda879b5940fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2512d256fe2466a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7251cfa33af4e1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7631,7 +7653,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb314b47f1c024891"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa579bbc547c4522"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7640,26 +7662,26 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22.219999313354492" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="28.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="7.78000020980835" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="36.66999816894531" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="10" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="40" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="27" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="9" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="38" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="38" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="44" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28.5" customHeight="1">
       <x:c r="A1" s="129" t="str">
-        <x:v>主流 AI 平台最新规格</x:v>
+        <x:v>主流 AI 平台规格与项目证据雷达</x:v>
       </x:c>
       <x:c r="B1" s="129"/>
       <x:c r="C1" s="129"/>
@@ -7678,7 +7700,7 @@
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
       <x:c r="A2" s="130" t="str">
-        <x:v>只使用官方页面；价格按表中口径，不同币种/峰谷不可直接横比。规格不等于小说质量。</x:v>
+        <x:v>仅记录各厂商官方当日规格；价格按未缓存/基准档。官方 benchmark、第三方 benchmark、项目实测严格分列，均不等于小说质量结论。</x:v>
       </x:c>
       <x:c r="B2" s="130"/>
       <x:c r="C2" s="130"/>
@@ -7735,7 +7757,7 @@
         <x:v>默认思考</x:v>
       </x:c>
       <x:c r="H4" s="169" t="str">
-        <x:v>平台能力</x:v>
+        <x:v>平台能力 / API caveat</x:v>
       </x:c>
       <x:c r="I4" s="169" t="str">
         <x:v>输入价/1M</x:v>
@@ -7747,19 +7769,19 @@
         <x:v>币种</x:v>
       </x:c>
       <x:c r="L4" s="169" t="str">
-        <x:v>价格/兼容 caveat</x:v>
+        <x:v>官方 benchmark</x:v>
       </x:c>
       <x:c r="M4" s="169" t="str">
-        <x:v>项目适配分</x:v>
+        <x:v>第三方 benchmark</x:v>
       </x:c>
       <x:c r="N4" s="169" t="str">
-        <x:v>建议角色</x:v>
+        <x:v>项目实测 / 建议角色</x:v>
       </x:c>
       <x:c r="O4" s="170" t="str">
-        <x:v>官方来源</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="51" customHeight="1">
+        <x:v>verified_at / 官方 URL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="96" customHeight="1">
       <x:c r="A5" s="171" t="str">
         <x:v>DeepSeek</x:v>
       </x:c>
@@ -7767,7 +7789,7 @@
         <x:v>deepseek-v4-flash</x:v>
       </x:c>
       <x:c r="C5" s="172" t="str">
-        <x:v>DeepSeek-V4-Flash-0731</x:v>
+        <x:v>DeepSeek-V4-Flash-0731（rolling ID）</x:v>
       </x:c>
       <x:c r="D5" s="184" t="n">
         <x:v>1000000</x:v>
@@ -7776,37 +7798,40 @@
         <x:v>384000</x:v>
       </x:c>
       <x:c r="F5" s="172" t="str">
-        <x:v>none/low/high/max；medium/xhigh→high</x:v>
+        <x:v>thinking disabled；low/high/max；medium/xhigh→high</x:v>
       </x:c>
       <x:c r="G5" s="172" t="str">
-        <x:v>thinking=enabled，effort=high</x:v>
+        <x:v>thinking enabled，effort=high</x:v>
       </x:c>
       <x:c r="H5" s="172" t="str">
-        <x:v>JSON、Tools、Responses、Anthropic</x:v>
+        <x:v>JSON Output、Tool Calls、Responses、Anthropic API、Web Search；thinking 下 temperature/top_p 无效；cache-hit 另计价</x:v>
       </x:c>
       <x:c r="I5" s="185" t="n">
-        <x:v>0.22</x:v>
+        <x:v>0.14</x:v>
       </x:c>
       <x:c r="J5" s="185" t="n">
-        <x:v>0.66</x:v>
+        <x:v>0.28</x:v>
       </x:c>
       <x:c r="K5" s="172" t="str">
         <x:v>USD</x:v>
       </x:c>
       <x:c r="L5" s="172" t="str">
-        <x:v>off-peak；peak 2x；thinking 下 temperature/top_p 无效</x:v>
-      </x:c>
-      <x:c r="M5" s="173" t="n">
-        <x:v>90</x:v>
+        <x:v>Code Agent：Terminal Bench 2.1 82.7、NL2Repo 54.2、DeepSWE 54.4（官方，max effort）；不是小说证据</x:v>
+      </x:c>
+      <x:c r="M5" s="194" t="str">
+        <x:v>未录入：尚无同一提示/同一裁判/可复现的小说对照</x:v>
       </x:c>
       <x:c r="N5" s="172" t="str">
-        <x:v>主默认候选；先修项目 route/effort</x:v>
+        <x:v>0 provider call；36-call 付费 pilot 只完成 dry-run/硬上限。低成本默认候选；首轮固定 high，max 只做难题对照</x:v>
       </x:c>
       <x:c r="O5" s="174" t="str">
-        <x:v>https://api-docs.deepseek.com/quick_start/pricing/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="51" customHeight="1">
+        <x:v>2026-09-01
+https://api-docs.deepseek.com/
+https://api-docs.deepseek.com/quick_start/pricing/
+https://api-docs.deepseek.com/updates/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="96" customHeight="1">
       <x:c r="A6" s="175" t="str">
         <x:v>DeepSeek</x:v>
       </x:c>
@@ -7814,7 +7839,7 @@
         <x:v>deepseek-v4-pro</x:v>
       </x:c>
       <x:c r="C6" s="176" t="str">
-        <x:v>DeepSeek-V4-Pro-0813</x:v>
+        <x:v>DeepSeek-V4-Pro-0813（rolling ID）</x:v>
       </x:c>
       <x:c r="D6" s="186" t="n">
         <x:v>1000000</x:v>
@@ -7823,37 +7848,39 @@
         <x:v>384000</x:v>
       </x:c>
       <x:c r="F6" s="176" t="str">
-        <x:v>none/low/high/max；medium/xhigh→high</x:v>
+        <x:v>thinking disabled；low/high/max；medium/xhigh→high</x:v>
       </x:c>
       <x:c r="G6" s="176" t="str">
-        <x:v>thinking=enabled，effort=high</x:v>
+        <x:v>thinking enabled，effort=high</x:v>
       </x:c>
       <x:c r="H6" s="176" t="str">
-        <x:v>JSON、Tools、Responses、Anthropic</x:v>
+        <x:v>JSON Output、Tool Calls、Responses、Anthropic API；thinking 下 temperature/top_p 无效；cache-hit 另计价</x:v>
       </x:c>
       <x:c r="I6" s="187" t="n">
-        <x:v>0.66</x:v>
+        <x:v>0.435</x:v>
       </x:c>
       <x:c r="J6" s="187" t="n">
-        <x:v>1.98</x:v>
+        <x:v>0.87</x:v>
       </x:c>
       <x:c r="K6" s="176" t="str">
         <x:v>USD</x:v>
       </x:c>
       <x:c r="L6" s="176" t="str">
-        <x:v>off-peak；peak 2x；高质量内容候选</x:v>
-      </x:c>
-      <x:c r="M6" s="177" t="n">
-        <x:v>88</x:v>
+        <x:v>未录入可与项目小说任务直接对应的官方指标</x:v>
+      </x:c>
+      <x:c r="M6" s="196" t="str">
+        <x:v>未录入：尚无同一提示/同一裁判/可复现的小说对照</x:v>
       </x:c>
       <x:c r="N6" s="176" t="str">
-        <x:v>写作/精修 A/B 候选</x:v>
+        <x:v>未运行。用于正文精修/语义审查 A/B 候选，不作默认批处理</x:v>
       </x:c>
       <x:c r="O6" s="178" t="str">
-        <x:v>https://api-docs.deepseek.com/guides/thinking_mode/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="51" customHeight="1">
+        <x:v>2026-09-01
+https://api-docs.deepseek.com/
+https://api-docs.deepseek.com/quick_start/pricing/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="96" customHeight="1">
       <x:c r="A7" s="175" t="str">
         <x:v>OpenAI</x:v>
       </x:c>
@@ -7861,7 +7888,7 @@
         <x:v>gpt-5.6-terra</x:v>
       </x:c>
       <x:c r="C7" s="176" t="str">
-        <x:v>GPT-5.6 Terra</x:v>
+        <x:v>GPT-5.6 Terra（平衡智能/成本）</x:v>
       </x:c>
       <x:c r="D7" s="186" t="n">
         <x:v>1050000</x:v>
@@ -7876,7 +7903,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="H7" s="176" t="str">
-        <x:v>Functions、Structured Outputs、Responses、Tools</x:v>
+        <x:v>Text+image input；Functions、Structured Outputs、Responses、Web/File Search、Code Interpreter、Computer Use；&gt;272K 全请求 input 2x/output 1.5x</x:v>
       </x:c>
       <x:c r="I7" s="187" t="n">
         <x:v>2</x:v>
@@ -7888,19 +7915,20 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="L7" s="176" t="str">
-        <x:v>&gt;272K 输入整请求 2x input/1.5x output</x:v>
-      </x:c>
-      <x:c r="M7" s="177" t="n">
-        <x:v>78</x:v>
+        <x:v>未录入小说任务官方 benchmark；“平衡智能/成本”只是官方定位</x:v>
+      </x:c>
+      <x:c r="M7" s="195" t="str">
+        <x:v>未录入：尚无同一提示/同一裁判/可复现的小说对照</x:v>
       </x:c>
       <x:c r="N7" s="176" t="str">
-        <x:v>平衡质量/成本的跨族 A/B</x:v>
+        <x:v>未运行。平衡质量/成本的跨族 A/B 候选</x:v>
       </x:c>
       <x:c r="O7" s="178" t="str">
-        <x:v>https://developers.openai.com/api/docs/models/gpt-5.6-terra</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="51" customHeight="1">
+        <x:v>2026-09-01
+https://developers.openai.com/api/docs/models/gpt-5.6-terra</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="96" customHeight="1">
       <x:c r="A8" s="175" t="str">
         <x:v>OpenAI</x:v>
       </x:c>
@@ -7908,7 +7936,7 @@
         <x:v>gpt-5.6-sol</x:v>
       </x:c>
       <x:c r="C8" s="176" t="str">
-        <x:v>GPT-5.6 Sol</x:v>
+        <x:v>GPT-5.6 Sol（复杂专业任务旗舰）</x:v>
       </x:c>
       <x:c r="D8" s="186" t="n">
         <x:v>1050000</x:v>
@@ -7917,13 +7945,13 @@
         <x:v>128000</x:v>
       </x:c>
       <x:c r="F8" s="176" t="str">
-        <x:v>none/low/medium/high/xhigh/max；pro mode</x:v>
+        <x:v>none/low/medium/high/xhigh/max</x:v>
       </x:c>
       <x:c r="G8" s="176" t="str">
         <x:v>medium</x:v>
       </x:c>
       <x:c r="H8" s="176" t="str">
-        <x:v>Functions、Structured Outputs、Responses、Tools</x:v>
+        <x:v>Text+image input；Functions、Structured Outputs、Responses、Web/File Search、Code Interpreter、Computer Use；&gt;272K 长输入阶梯价</x:v>
       </x:c>
       <x:c r="I8" s="187" t="n">
         <x:v>4</x:v>
@@ -7935,19 +7963,20 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="L8" s="176" t="str">
-        <x:v>旗舰；复杂审查/高价值任务</x:v>
-      </x:c>
-      <x:c r="M8" s="177" t="n">
-        <x:v>75</x:v>
+        <x:v>未录入小说任务官方 benchmark；旗舰定位不作项目质量证明</x:v>
+      </x:c>
+      <x:c r="M8" s="196" t="str">
+        <x:v>未录入：尚无同一提示/同一裁判/可复现的小说对照</x:v>
       </x:c>
       <x:c r="N8" s="176" t="str">
-        <x:v>高难审查/结构验证 A/B</x:v>
+        <x:v>未运行。高难结构/最终审计 A/B，不作默认</x:v>
       </x:c>
       <x:c r="O8" s="178" t="str">
-        <x:v>https://developers.openai.com/api/docs/models/gpt-5.6-sol</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="51" customHeight="1">
+        <x:v>2026-09-01
+https://developers.openai.com/api/docs/models/gpt-5.6-sol</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="96" customHeight="1">
       <x:c r="A9" s="175" t="str">
         <x:v>Anthropic</x:v>
       </x:c>
@@ -7964,13 +7993,13 @@
         <x:v>128000</x:v>
       </x:c>
       <x:c r="F9" s="176" t="str">
-        <x:v>adaptive thinking + effort</x:v>
+        <x:v>adaptive thinking；low/medium/high/xhigh/max effort</x:v>
       </x:c>
       <x:c r="G9" s="176" t="str">
-        <x:v>thinking on，effort high</x:v>
+        <x:v>adaptive on，effort=high</x:v>
       </x:c>
       <x:c r="H9" s="176" t="str">
-        <x:v>Tools、Files/PDF、Vision、Structured Outputs</x:v>
+        <x:v>Tools、Files/PDF、Vision、Structured Outputs；非默认 temperature/top_p/top_k 返回 400；新 tokenizer 同文约 +30% tokens</x:v>
       </x:c>
       <x:c r="I9" s="187" t="n">
         <x:v>2</x:v>
@@ -7982,19 +8011,21 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="L9" s="176" t="str">
-        <x:v>非默认 temperature/top_p/top_k 返回 400；新 tokenizer 同文约多 30% token</x:v>
-      </x:c>
-      <x:c r="M9" s="177" t="n">
-        <x:v>72</x:v>
+        <x:v>官方称相比 4.6 提升 coding/agentic；本表不把该定位换算成小说分数</x:v>
+      </x:c>
+      <x:c r="M9" s="195" t="str">
+        <x:v>未录入：尚无同一提示/同一裁判/可复现的小说对照</x:v>
       </x:c>
       <x:c r="N9" s="176" t="str">
-        <x:v>内容/审查强候选；必须按模型抑制采样参数</x:v>
+        <x:v>未运行。内容/审查强候选；接入前必须按模型抑制采样参数</x:v>
       </x:c>
       <x:c r="O9" s="178" t="str">
-        <x:v>https://platform.claude.com/docs/en/models/sonnet-5/whats-new-sonnet-5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="51" customHeight="1">
+        <x:v>2026-09-01
+https://platform.claude.com/docs/en/models/sonnet-5/whats-new-sonnet-5
+https://platform.claude.com/docs/en/build-with-claude/effort</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="96" customHeight="1">
       <x:c r="A10" s="175" t="str">
         <x:v>Anthropic</x:v>
       </x:c>
@@ -8011,13 +8042,13 @@
         <x:v>128000</x:v>
       </x:c>
       <x:c r="F10" s="176" t="str">
-        <x:v>adaptive thinking + effort</x:v>
+        <x:v>adaptive thinking；low/medium/high/xhigh/max effort</x:v>
       </x:c>
       <x:c r="G10" s="176" t="str">
-        <x:v>thinking on，effort high</x:v>
+        <x:v>adaptive on，effort=high</x:v>
       </x:c>
       <x:c r="H10" s="176" t="str">
-        <x:v>Tools、long-horizon、Vision</x:v>
+        <x:v>Tools、Vision、long-horizon agentic；max_tokens 同时约束 thinking+回答；effort 为软指引</x:v>
       </x:c>
       <x:c r="I10" s="187" t="n">
         <x:v>5</x:v>
@@ -8029,19 +8060,21 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="L10" s="176" t="str">
-        <x:v>高成本；适合少量高价值裁决</x:v>
-      </x:c>
-      <x:c r="M10" s="177" t="n">
-        <x:v>66</x:v>
+        <x:v>官方定位为复杂 agentic/企业工作；未录入小说专项指标</x:v>
+      </x:c>
+      <x:c r="M10" s="196" t="str">
+        <x:v>未录入：尚无同一提示/同一裁判/可复现的小说对照</x:v>
       </x:c>
       <x:c r="N10" s="176" t="str">
-        <x:v>最终审计 A/B，不作默认批处理</x:v>
+        <x:v>未运行。最终高价值裁决 A/B，不作默认批处理</x:v>
       </x:c>
       <x:c r="O10" s="178" t="str">
-        <x:v>https://platform.claude.com/docs/en/about-claude/models/whats-new-claude-4-6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="51" customHeight="1">
+        <x:v>2026-09-01
+https://platform.claude.com/docs/en/about-claude/models/choosing-a-model
+https://platform.claude.com/docs/en/build-with-claude/effort</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="96" customHeight="1">
       <x:c r="A11" s="175" t="str">
         <x:v>Google</x:v>
       </x:c>
@@ -8049,7 +8082,7 @@
         <x:v>gemini-3.7-flash</x:v>
       </x:c>
       <x:c r="C11" s="176" t="str">
-        <x:v>Gemini 3.7 Flash</x:v>
+        <x:v>Gemini 3.7 Flash（GA）</x:v>
       </x:c>
       <x:c r="D11" s="186" t="n">
         <x:v>1048576</x:v>
@@ -8058,13 +8091,13 @@
         <x:v>65536</x:v>
       </x:c>
       <x:c r="F11" s="176" t="str">
-        <x:v>low/medium/high</x:v>
+        <x:v>low/medium/high；minimal 报错</x:v>
       </x:c>
       <x:c r="G11" s="176" t="str">
         <x:v>medium</x:v>
       </x:c>
       <x:c r="H11" s="176" t="str">
-        <x:v>多模态、Tools、Search/Maps、Structured Outputs</x:v>
+        <x:v>多模态、Function Calling、Structured Outputs、Search/Maps、Code Execution、Computer Use；采样参数迁移有兼容变化；价格为 2026 年底前介绍价</x:v>
       </x:c>
       <x:c r="I11" s="187" t="n">
         <x:v>0.75</x:v>
@@ -8076,19 +8109,22 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="L11" s="176" t="str">
-        <x:v>2026-12-31 前介绍价；采样参数迁移有兼容变化</x:v>
-      </x:c>
-      <x:c r="M11" s="177" t="n">
-        <x:v>80</x:v>
+        <x:v>官方定位为 coding/agentic/multimodal workhorse；未录入小说专项分数</x:v>
+      </x:c>
+      <x:c r="M11" s="195" t="str">
+        <x:v>未录入：尚无同一提示/同一裁判/可复现的小说对照</x:v>
       </x:c>
       <x:c r="N11" s="176" t="str">
-        <x:v>长上下文/多模态/结构 A/B</x:v>
+        <x:v>未运行。长上下文/多模态/结构化 A/B 候选</x:v>
       </x:c>
       <x:c r="O11" s="178" t="str">
-        <x:v>https://ai.google.dev/gemini-api/docs/models/gemini-3.7-flash</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="51" customHeight="1">
+        <x:v>2026-09-01
+https://ai.google.dev/gemini-api/docs/latest-model
+https://ai.google.dev/gemini-api/docs/models/gemini-3.7-flash
+https://ai.google.dev/gemini-api/docs/pricing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="96" customHeight="1">
       <x:c r="A12" s="179" t="str">
         <x:v>Alibaba</x:v>
       </x:c>
@@ -8105,13 +8141,13 @@
         <x:v>131072</x:v>
       </x:c>
       <x:c r="F12" s="180" t="str">
-        <x:v>hybrid thinking；thinking_budget/Responses effort</x:v>
+        <x:v>hybrid thinking；enable_thinking/thinking_budget；Responses reasoning.effort</x:v>
       </x:c>
       <x:c r="G12" s="180" t="str">
-        <x:v>thinking enabled</x:v>
+        <x:v>thinking enabled/adaptive</x:v>
       </x:c>
       <x:c r="H12" s="180" t="str">
-        <x:v>Function Calling、Built-in Tools、Structured Output</x:v>
+        <x:v>Function Calling、Built-in Tools、Structured Output、Context Cache；北京基准价仅 &lt;=256K，&gt;256K 为 6/24 CNY</x:v>
       </x:c>
       <x:c r="I12" s="189" t="n">
         <x:v>2</x:v>
@@ -8123,16 +8159,19 @@
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="L12" s="180" t="str">
-        <x:v>北京 &lt;=256K 原价；&gt;256K 为 6/24 CNY</x:v>
-      </x:c>
-      <x:c r="M12" s="181" t="n">
-        <x:v>82</x:v>
+        <x:v>官方建议非编码办公任务从 3.7 Plus 起步；未录入小说专项分数</x:v>
+      </x:c>
+      <x:c r="M12" s="197" t="str">
+        <x:v>未录入：尚无同一提示/同一裁判/可复现的小说对照</x:v>
       </x:c>
       <x:c r="N12" s="180" t="str">
-        <x:v>中文长篇与结构化 A/B</x:v>
+        <x:v>未运行。中文长篇/结构化 A/B 候选；跨币种成本不直接排名</x:v>
       </x:c>
       <x:c r="O12" s="182" t="str">
-        <x:v>https://help.aliyun.com/zh/model-studio/qwen3-7-plus</x:v>
+        <x:v>2026-09-01
+https://help.aliyun.com/zh/model-studio/qwen3-7-plus
+https://help.aliyun.com/en/model-studio/model-pricing
+https://help.aliyun.com/en/model-studio/text-generation-model/</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8154,7 +8193,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra39fed1370d34b97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d8c56d15a0b4068"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8474,7 +8513,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8d2b58f5ec042a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95eb376f8ef6429e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8877,7 +8916,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf17cc7db3c94476e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f5a5b94201d4f1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9360,7 +9399,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e11409df1454245"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1733fe8c2d94954"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>